<commit_message>
Excel export: keep printed '=' text as text, not formulas; internal sheet links
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MKgSdDvVSCL7zgQ1r4fLnk
</commit_message>
<xml_diff>
--- a/downloads/korea-1929-30-tables.xlsx
+++ b/downloads/korea-1929-30-tables.xlsx
@@ -1849,54 +1849,54 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A37" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A38" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A39" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A40" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A41" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A42" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A43" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A44" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A45" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A46" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A47" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A48" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A49" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A50" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A51" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A52" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A53" r:id="rId48"/>
+    <hyperlink ref="A6" location="'p0026_1'!A1"/>
+    <hyperlink ref="A7" location="'p0029_1'!A1"/>
+    <hyperlink ref="A8" location="'p0029_2'!A1"/>
+    <hyperlink ref="A9" location="'p0031_1'!A1"/>
+    <hyperlink ref="A10" location="'p0033_1'!A1"/>
+    <hyperlink ref="A11" location="'p0059_1'!A1"/>
+    <hyperlink ref="A12" location="'p0060_1'!A1"/>
+    <hyperlink ref="A13" location="'p0064_1'!A1"/>
+    <hyperlink ref="A14" location="'p0065_1'!A1"/>
+    <hyperlink ref="A15" location="'p0068_1'!A1"/>
+    <hyperlink ref="A16" location="'p0070_1'!A1"/>
+    <hyperlink ref="A17" location="'p0071_1'!A1"/>
+    <hyperlink ref="A18" location="'p0072_1'!A1"/>
+    <hyperlink ref="A19" location="'p0075_1'!A1"/>
+    <hyperlink ref="A20" location="'p0076_1'!A1"/>
+    <hyperlink ref="A21" location="'p0078_1'!A1"/>
+    <hyperlink ref="A22" location="'p0079_1'!A1"/>
+    <hyperlink ref="A23" location="'p0080_1'!A1"/>
+    <hyperlink ref="A24" location="'p0081_1'!A1"/>
+    <hyperlink ref="A25" location="'p0081_2'!A1"/>
+    <hyperlink ref="A26" location="'p0087_1'!A1"/>
+    <hyperlink ref="A27" location="'p0091_1'!A1"/>
+    <hyperlink ref="A28" location="'p0103_1'!A1"/>
+    <hyperlink ref="A29" location="'p0107_1'!A1"/>
+    <hyperlink ref="A30" location="'p0123_1'!A1"/>
+    <hyperlink ref="A31" location="'p0126_1'!A1"/>
+    <hyperlink ref="A32" location="'p0128_1'!A1"/>
+    <hyperlink ref="A33" location="'p0133_1'!A1"/>
+    <hyperlink ref="A34" location="'p0137_1'!A1"/>
+    <hyperlink ref="A35" location="'p0140_1'!A1"/>
+    <hyperlink ref="A36" location="'p0141_1'!A1"/>
+    <hyperlink ref="A37" location="'p0142_1'!A1"/>
+    <hyperlink ref="A38" location="'p0143_1'!A1"/>
+    <hyperlink ref="A39" location="'p0144_1'!A1"/>
+    <hyperlink ref="A40" location="'p0144_2'!A1"/>
+    <hyperlink ref="A41" location="'p0147_1'!A1"/>
+    <hyperlink ref="A42" location="'p0148_1'!A1"/>
+    <hyperlink ref="A43" location="'p0158_1'!A1"/>
+    <hyperlink ref="A44" location="'p0160_1'!A1"/>
+    <hyperlink ref="A45" location="'p0164_1'!A1"/>
+    <hyperlink ref="A46" location="'p0174_1'!A1"/>
+    <hyperlink ref="A47" location="'p0179_1'!A1"/>
+    <hyperlink ref="A48" location="'p0181_1'!A1"/>
+    <hyperlink ref="A49" location="'p0182_1'!A1"/>
+    <hyperlink ref="A50" location="'p0182_2'!A1"/>
+    <hyperlink ref="A51" location="'p0185_1'!A1"/>
+    <hyperlink ref="A52" location="'p0185_2'!A1"/>
+    <hyperlink ref="A53" location="'p0187_1'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2121,7 +2121,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2508,7 +2508,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2702,7 +2702,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2884,7 +2884,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3190,7 +3190,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3493,7 +3493,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3984,7 +3984,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4281,7 +4281,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4824,7 +4824,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5220,7 +5220,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5557,7 +5557,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5991,7 +5991,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6553,7 +6553,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7118,7 +7118,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7790,7 +7790,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
+    <hyperlink ref="A4" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8314,7 +8314,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8567,7 +8567,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8952,7 +8952,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9443,7 +9443,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9757,7 +9757,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9918,7 +9918,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10567,7 +10567,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10820,7 +10820,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11050,7 +11050,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11235,7 +11235,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11431,7 +11431,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11592,7 +11592,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11745,7 +11745,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11884,7 +11884,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12070,7 +12070,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12300,7 +12300,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12460,7 +12460,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
+    <hyperlink ref="A4" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14086,7 +14086,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14308,7 +14308,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14630,7 +14630,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14935,7 +14935,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15474,7 +15474,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15674,7 +15674,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15818,7 +15818,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16586,7 +16586,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16747,7 +16747,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17338,7 +17338,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17542,7 +17542,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17903,7 +17903,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -18088,7 +18088,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -18595,7 +18595,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19616,7 +19616,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -20057,7 +20057,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>